<commit_message>
excel update 2026-06-23 14:44
</commit_message>
<xml_diff>
--- a/order_result.xlsx
+++ b/order_result.xlsx
@@ -11,7 +11,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'발주확인대상'!$A$1:$K$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'발주확인대상'!$A$1:$K$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K120"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4058,956 +4058,848 @@
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B75" s="7" t="n">
-        <v>7000194</v>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>아사콜관장액 4그람/100밀리리터 7병(메살라진)</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>2,4</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-09</t>
-        </is>
-      </c>
-      <c r="F75" s="7" t="inlineStr">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="n">
+        <v>1300750</v>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>OPADRY 03B44038 Pink(인도,별규)</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>2023-02-09</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="8" t="n">
+        <v>1230</v>
+      </c>
+      <c r="H75" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="I75" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K75" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>1300261</v>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Benfotiamine(KP,Bioxera)</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>2023-02-15</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>1224</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K76" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="n">
+        <v>1000028</v>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Erdosteine(Interquim)</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>2023-03-08</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>1203</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>18239.7</v>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K77" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="n">
+        <v>1001252</v>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>DL-α-Tocopherol Acetate</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>2023-10-18</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="G78" s="8" t="n">
+        <v>979</v>
+      </c>
+      <c r="H78" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K78" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="n">
+        <v>1000336</v>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Minocycline Hydrochloride</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>7,8</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="G79" s="8" t="n">
+        <v>811</v>
+      </c>
+      <c r="H79" s="8" t="n">
+        <v>865.9</v>
+      </c>
+      <c r="I79" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K79" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="n">
+        <v>1000178</v>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>Benfotiamine(Hamari, KP)</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>2024-08-07</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="n">
+        <v>292</v>
+      </c>
+      <c r="G80" s="8" t="n">
+        <v>685</v>
+      </c>
+      <c r="H80" s="8" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I80" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K80" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="n">
+        <v>1300593</v>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Opadry clear 06A29148(별규,Colorcon)</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I75" s="7" t="n">
-        <v>34252</v>
-      </c>
-      <c r="J75" s="7" t="inlineStr">
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>2024-08-08</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="n">
+        <v>423</v>
+      </c>
+      <c r="G81" s="8" t="n">
+        <v>684</v>
+      </c>
+      <c r="H81" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="I81" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K81" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="n">
+        <v>1000354</v>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Oseltamivir phosphate</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K75" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="n">
-        <v>7000196</v>
-      </c>
-      <c r="C76" s="7" t="inlineStr">
-        <is>
-          <t>아사콜좌약500밀리그람(메살라진) 20 Supp.</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E76" s="7" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
-      <c r="F76" s="7" t="inlineStr">
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>2024-08-30</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="n">
+        <v>266</v>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>662</v>
+      </c>
+      <c r="H82" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I82" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K82" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="n">
+        <v>1300180</v>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Opadry QX 321A130006 Orange(칼라콘,별규)</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>2024-10-08</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="n">
+        <v>153</v>
+      </c>
+      <c r="G83" s="8" t="n">
+        <v>623</v>
+      </c>
+      <c r="H83" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I83" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K83" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="n">
+        <v>1000378</v>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Opadry AMB yellow 80W220002</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>89180</v>
-      </c>
-      <c r="J76" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K76" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B77" s="7" t="n">
-        <v>7000304</v>
-      </c>
-      <c r="C77" s="7" t="inlineStr">
-        <is>
-          <t>다이아벡스XR 서방정 500mg 60T</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="E77" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I77" s="7" t="n">
-        <v>560000</v>
-      </c>
-      <c r="J77" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K77" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B78" s="7" t="n">
-        <v>7000305</v>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>다이아벡스XR 서방정 1000MG 60T</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="F78" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I78" s="7" t="n">
-        <v>530000</v>
-      </c>
-      <c r="J78" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K78" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B79" s="7" t="n">
-        <v>7000775</v>
-      </c>
-      <c r="C79" s="7" t="inlineStr">
-        <is>
-          <t>엔토코트(Budesonide 2.3mg) 7정</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="n">
+        <v>230</v>
+      </c>
+      <c r="G84" s="8" t="n">
+        <v>587</v>
+      </c>
+      <c r="H84" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="I84" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K84" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="n">
+        <v>1000061</v>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Opadry 03B54445 Pink(Colorcon)</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>2024-11-21</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="G85" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="H85" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="I85" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K85" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="n">
+        <v>1001238</v>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Minocycline Hydrochloride(Cipan)</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>2024-11-28</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G86" s="8" t="n">
+        <v>572</v>
+      </c>
+      <c r="H86" s="8" t="n">
+        <v>717.5</v>
+      </c>
+      <c r="I86" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K86" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="n">
+        <v>1301736</v>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Ampicillin sodium(USP, Shandong Lukang)</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>533</v>
+      </c>
+      <c r="H87" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="I87" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K87" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="n">
+        <v>1300178</v>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Opadry QX 321A120004 Yellow(칼라콘,In-house</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I79" s="7" t="n">
-        <v>6000</v>
-      </c>
-      <c r="J79" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K79" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="n">
-        <v>7000791</v>
-      </c>
-      <c r="C80" s="7" t="inlineStr">
-        <is>
-          <t>글루리아드정 500/2.5mg 60TT(소포장)</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-05</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="n">
+        <v>216</v>
+      </c>
+      <c r="G88" s="8" t="n">
+        <v>503</v>
+      </c>
+      <c r="H88" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I88" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K88" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="n">
+        <v>1301757</v>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Human serum albumin(20%)(Octapharma)</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E80" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I80" s="7" t="n">
-        <v>18000</v>
-      </c>
-      <c r="J80" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K80" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B81" s="7" t="n">
-        <v>7000793</v>
-      </c>
-      <c r="C81" s="7" t="inlineStr">
-        <is>
-          <t>글루리아드정 500/5mg 60TT(소포장)</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="8" t="n">
+        <v>491</v>
+      </c>
+      <c r="H89" s="8" t="n">
+        <v>61000</v>
+      </c>
+      <c r="I89" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K89" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="n">
+        <v>1001226</v>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Dried Ginseng Ext(GUANGDONG)</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G81" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H81" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I81" s="7" t="n">
-        <v>9500</v>
-      </c>
-      <c r="J81" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K81" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="n">
-        <v>7000794</v>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>글루리아드정 500/5mg 120TT</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr">
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-21</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="n">
+        <v>257</v>
+      </c>
+      <c r="G90" s="8" t="n">
+        <v>487</v>
+      </c>
+      <c r="H90" s="8" t="n">
+        <v>2250</v>
+      </c>
+      <c r="I90" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K90" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="n">
+        <v>1001173</v>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>오파드라이 노란색 (03B62323)</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E82" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="F82" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H82" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I82" s="7" t="n">
-        <v>9500</v>
-      </c>
-      <c r="J82" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K82" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B83" s="7" t="n">
-        <v>7000800</v>
-      </c>
-      <c r="C83" s="7" t="inlineStr">
-        <is>
-          <t>인스타닐나잘스프레이 100㎍ 1병(펜타닐시트르산염)</t>
-        </is>
-      </c>
-      <c r="D83" s="7" t="inlineStr">
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-25</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="G91" s="8" t="n">
+        <v>483</v>
+      </c>
+      <c r="H91" s="8" t="n">
+        <v>275</v>
+      </c>
+      <c r="I91" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K91" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>⚪ 발주중단의심</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="n">
+        <v>1301404</v>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>OPADRY® AMB II 88A150017 RED(별규,칼라콘)</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E83" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="F83" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I83" s="7" t="n">
-        <v>17000</v>
-      </c>
-      <c r="J83" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K83" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B84" s="7" t="n">
-        <v>7000801</v>
-      </c>
-      <c r="C84" s="7" t="inlineStr">
-        <is>
-          <t>인스타닐나잘스프레이 200㎍ 1병(펜타닐시트르산염)</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="F84" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I84" s="7" t="n">
-        <v>6000</v>
-      </c>
-      <c r="J84" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K84" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B85" s="7" t="n">
-        <v>7000802</v>
-      </c>
-      <c r="C85" s="7" t="inlineStr">
-        <is>
-          <t>인스타닐나잘스프레이 50㎍ 1병(펜타닐시트르산염)</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H85" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I85" s="7" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J85" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K85" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="n">
-        <v>7300174</v>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>스타빅현탁액 20mL 100PP(20포X5EA)</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="E86" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-10</t>
-        </is>
-      </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I86" s="7" t="n">
-        <v>149500</v>
-      </c>
-      <c r="J86" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K86" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B87" s="7" t="n">
-        <v>7300175</v>
-      </c>
-      <c r="C87" s="7" t="inlineStr">
-        <is>
-          <t>스타빅현탁액 20mL 72PP(6포X12EA)</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-10</t>
-        </is>
-      </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H87" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I87" s="7" t="n">
-        <v>18800</v>
-      </c>
-      <c r="J87" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K87" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="n">
-        <v>7300176</v>
-      </c>
-      <c r="C88" s="7" t="inlineStr">
-        <is>
-          <t>스타빅현탁액 500ML</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E88" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-10</t>
-        </is>
-      </c>
-      <c r="F88" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G88" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H88" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I88" s="7" t="n">
-        <v>11000</v>
-      </c>
-      <c r="J88" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K88" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B89" s="7" t="n">
-        <v>8000037</v>
-      </c>
-      <c r="C89" s="7" t="inlineStr">
-        <is>
-          <t>올메텍정 20mg 반제품</t>
-        </is>
-      </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E89" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H89" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I89" s="7" t="n">
-        <v>29900000</v>
-      </c>
-      <c r="J89" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K89" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B90" s="7" t="n">
-        <v>8000047</v>
-      </c>
-      <c r="C90" s="7" t="inlineStr">
-        <is>
-          <t>올메텍플러스정 반제품</t>
-        </is>
-      </c>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E90" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="F90" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G90" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H90" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I90" s="7" t="n">
-        <v>12600000</v>
-      </c>
-      <c r="J90" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K90" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="n">
-        <v>8000052</v>
-      </c>
-      <c r="C91" s="7" t="inlineStr">
-        <is>
-          <t>올메텍정 40mg 반제품</t>
-        </is>
-      </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E91" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H91" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I91" s="7" t="n">
-        <v>3190000</v>
-      </c>
-      <c r="J91" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K91" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>🆕 신규품목</t>
-        </is>
-      </c>
-      <c r="B92" s="7" t="n">
-        <v>8000901</v>
-      </c>
-      <c r="C92" s="7" t="inlineStr">
-        <is>
-          <t>올메텍정 10mg 반제품</t>
-        </is>
-      </c>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="F92" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H92" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I92" s="7" t="n">
-        <v>27500000</v>
-      </c>
-      <c r="J92" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K92" s="7" t="inlineStr">
-        <is>
-          <t>과거 3개년 이력 없는 신규 품목</t>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="H92" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="I92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K92" s="8" t="inlineStr">
+        <is>
+          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
     </row>
@@ -5018,31 +4910,31 @@
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>1300750</v>
+        <v>1000157</v>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>OPADRY 03B44038 Pink(인도,별규)</t>
+          <t>Agar</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>2023-02-09</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="F93" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G93" s="8" t="n">
-        <v>1230</v>
+        <v>469</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I93" s="8" t="n">
         <v>0</v>
@@ -5065,31 +4957,31 @@
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>1300261</v>
+        <v>1300542</v>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Benfotiamine(KP,Bioxera)</t>
+          <t>Opadry Yellow 03F620190(IH,Colorcon)</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>2023-02-15</t>
+          <t>2025-03-18</t>
         </is>
       </c>
       <c r="F94" s="8" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="G94" s="8" t="n">
-        <v>1224</v>
+        <v>462</v>
       </c>
       <c r="H94" s="8" t="n">
-        <v>6000</v>
+        <v>100</v>
       </c>
       <c r="I94" s="8" t="n">
         <v>0</v>
@@ -5112,31 +5004,31 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>1000028</v>
+        <v>1300181</v>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Erdosteine(Interquim)</t>
+          <t>Opadry QX 321A120007 Yellow(칼라콘,별규)</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>1,3</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>2023-03-08</t>
+          <t>2025-03-25</t>
         </is>
       </c>
       <c r="F95" s="8" t="n">
-        <v>8</v>
+        <v>391</v>
       </c>
       <c r="G95" s="8" t="n">
-        <v>1203</v>
+        <v>455</v>
       </c>
       <c r="H95" s="8" t="n">
-        <v>18239.7</v>
+        <v>100</v>
       </c>
       <c r="I95" s="8" t="n">
         <v>0</v>
@@ -5159,28 +5051,28 @@
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>1001252</v>
+        <v>1000202</v>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>DL-α-Tocopherol Acetate</t>
+          <t>0.1% Cyanocobalamin(Ningxia)</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>2023-10-18</t>
+          <t>2025-04-14</t>
         </is>
       </c>
       <c r="F96" s="8" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="G96" s="8" t="n">
-        <v>979</v>
+        <v>435</v>
       </c>
       <c r="H96" s="8" t="n">
         <v>1500</v>
@@ -5206,31 +5098,31 @@
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>1000336</v>
+        <v>1000367</v>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Minocycline Hydrochloride</t>
+          <t>Opadry OY-S-29019</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>7,8</t>
+          <t>3,4</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>2025-04-15</t>
         </is>
       </c>
       <c r="F97" s="8" t="n">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="G97" s="8" t="n">
-        <v>811</v>
+        <v>434</v>
       </c>
       <c r="H97" s="8" t="n">
-        <v>865.9</v>
+        <v>133.3</v>
       </c>
       <c r="I97" s="8" t="n">
         <v>0</v>
@@ -5253,31 +5145,31 @@
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>1000178</v>
+        <v>1301203</v>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Benfotiamine(Hamari, KP)</t>
+          <t>Opadry AMB II 88A610005 GREEN (별규,칼라콘)</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>2024-08-07</t>
+          <t>2025-04-16</t>
         </is>
       </c>
       <c r="F98" s="8" t="n">
-        <v>292</v>
+        <v>70</v>
       </c>
       <c r="G98" s="8" t="n">
-        <v>685</v>
+        <v>433</v>
       </c>
       <c r="H98" s="8" t="n">
-        <v>4000</v>
+        <v>175</v>
       </c>
       <c r="I98" s="8" t="n">
         <v>0</v>
@@ -5300,31 +5192,31 @@
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>1300593</v>
+        <v>1300614</v>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Opadry clear 06A29148(별규,Colorcon)</t>
+          <t>Human serum albumin(세관폐기)</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,4</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>2025-04-28</t>
         </is>
       </c>
       <c r="F99" s="8" t="n">
-        <v>423</v>
+        <v>75</v>
       </c>
       <c r="G99" s="8" t="n">
-        <v>684</v>
+        <v>421</v>
       </c>
       <c r="H99" s="8" t="n">
-        <v>125</v>
+        <v>31200</v>
       </c>
       <c r="I99" s="8" t="n">
         <v>0</v>
@@ -5347,31 +5239,31 @@
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>1000354</v>
+        <v>1300949</v>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Oseltamivir phosphate</t>
+          <t>Opadry Pink 03F640111(IH,칼라콘)</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2025-04-28</t>
         </is>
       </c>
       <c r="F100" s="8" t="n">
-        <v>266</v>
+        <v>0</v>
       </c>
       <c r="G100" s="8" t="n">
-        <v>662</v>
+        <v>421</v>
       </c>
       <c r="H100" s="8" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I100" s="8" t="n">
         <v>0</v>
@@ -5394,31 +5286,31 @@
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>1300180</v>
+        <v>1301322</v>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Opadry QX 321A130006 Orange(칼라콘,별규)</t>
+          <t>Oxymetazoline HCl(USP,CTX)</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>2024-10-08</t>
+          <t>2025-04-30</t>
         </is>
       </c>
       <c r="F101" s="8" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="G101" s="8" t="n">
-        <v>623</v>
+        <v>419</v>
       </c>
       <c r="H101" s="8" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="I101" s="8" t="n">
         <v>0</v>
@@ -5441,31 +5333,31 @@
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>1000378</v>
+        <v>1300438</v>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Opadry AMB yellow 80W220002</t>
+          <t>오파드라이 20A680000 칼라콘</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2025-05-29</t>
         </is>
       </c>
       <c r="F102" s="8" t="n">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="G102" s="8" t="n">
-        <v>587</v>
+        <v>390</v>
       </c>
       <c r="H102" s="8" t="n">
-        <v>200</v>
+        <v>62.5</v>
       </c>
       <c r="I102" s="8" t="n">
         <v>0</v>
@@ -5481,854 +5373,8 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B103" s="8" t="n">
-        <v>1000061</v>
-      </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
-          <t>Opadry 03B54445 Pink(Colorcon)</t>
-        </is>
-      </c>
-      <c r="D103" s="8" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E103" s="8" t="inlineStr">
-        <is>
-          <t>2024-11-21</t>
-        </is>
-      </c>
-      <c r="F103" s="8" t="n">
-        <v>180</v>
-      </c>
-      <c r="G103" s="8" t="n">
-        <v>579</v>
-      </c>
-      <c r="H103" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="I103" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K103" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B104" s="8" t="n">
-        <v>1001238</v>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t>Minocycline Hydrochloride(Cipan)</t>
-        </is>
-      </c>
-      <c r="D104" s="8" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E104" s="8" t="inlineStr">
-        <is>
-          <t>2024-11-28</t>
-        </is>
-      </c>
-      <c r="F104" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="G104" s="8" t="n">
-        <v>572</v>
-      </c>
-      <c r="H104" s="8" t="n">
-        <v>717.5</v>
-      </c>
-      <c r="I104" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K104" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B105" s="8" t="n">
-        <v>1301736</v>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t>Ampicillin sodium(USP, Shandong Lukang)</t>
-        </is>
-      </c>
-      <c r="D105" s="8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>2025-01-06</t>
-        </is>
-      </c>
-      <c r="F105" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" s="8" t="n">
-        <v>533</v>
-      </c>
-      <c r="H105" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="I105" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J105" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K105" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="18" customHeight="1">
-      <c r="A106" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B106" s="8" t="n">
-        <v>1300178</v>
-      </c>
-      <c r="C106" s="8" t="inlineStr">
-        <is>
-          <t>Opadry QX 321A120004 Yellow(칼라콘,In-house</t>
-        </is>
-      </c>
-      <c r="D106" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E106" s="8" t="inlineStr">
-        <is>
-          <t>2025-02-05</t>
-        </is>
-      </c>
-      <c r="F106" s="8" t="n">
-        <v>216</v>
-      </c>
-      <c r="G106" s="8" t="n">
-        <v>503</v>
-      </c>
-      <c r="H106" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="I106" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J106" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K106" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B107" s="8" t="n">
-        <v>1301757</v>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>Human serum albumin(20%)(Octapharma)</t>
-        </is>
-      </c>
-      <c r="D107" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E107" s="8" t="inlineStr">
-        <is>
-          <t>2025-02-17</t>
-        </is>
-      </c>
-      <c r="F107" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" s="8" t="n">
-        <v>491</v>
-      </c>
-      <c r="H107" s="8" t="n">
-        <v>61000</v>
-      </c>
-      <c r="I107" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J107" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K107" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B108" s="8" t="n">
-        <v>1001226</v>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>Dried Ginseng Ext(GUANGDONG)</t>
-        </is>
-      </c>
-      <c r="D108" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E108" s="8" t="inlineStr">
-        <is>
-          <t>2025-02-21</t>
-        </is>
-      </c>
-      <c r="F108" s="8" t="n">
-        <v>257</v>
-      </c>
-      <c r="G108" s="8" t="n">
-        <v>487</v>
-      </c>
-      <c r="H108" s="8" t="n">
-        <v>2250</v>
-      </c>
-      <c r="I108" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K108" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="18" customHeight="1">
-      <c r="A109" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B109" s="8" t="n">
-        <v>1001173</v>
-      </c>
-      <c r="C109" s="8" t="inlineStr">
-        <is>
-          <t>오파드라이 노란색 (03B62323)</t>
-        </is>
-      </c>
-      <c r="D109" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E109" s="8" t="inlineStr">
-        <is>
-          <t>2025-02-25</t>
-        </is>
-      </c>
-      <c r="F109" s="8" t="n">
-        <v>63</v>
-      </c>
-      <c r="G109" s="8" t="n">
-        <v>483</v>
-      </c>
-      <c r="H109" s="8" t="n">
-        <v>275</v>
-      </c>
-      <c r="I109" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J109" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K109" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B110" s="8" t="n">
-        <v>1301404</v>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
-          <t>OPADRY® AMB II 88A150017 RED(별규,칼라콘)</t>
-        </is>
-      </c>
-      <c r="D110" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E110" s="8" t="inlineStr">
-        <is>
-          <t>2025-02-28</t>
-        </is>
-      </c>
-      <c r="F110" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G110" s="8" t="n">
-        <v>480</v>
-      </c>
-      <c r="H110" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="I110" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J110" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K110" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B111" s="8" t="n">
-        <v>1000157</v>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t>Agar</t>
-        </is>
-      </c>
-      <c r="D111" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E111" s="8" t="inlineStr">
-        <is>
-          <t>2025-03-11</t>
-        </is>
-      </c>
-      <c r="F111" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" s="8" t="n">
-        <v>469</v>
-      </c>
-      <c r="H111" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="I111" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K111" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B112" s="8" t="n">
-        <v>1300542</v>
-      </c>
-      <c r="C112" s="8" t="inlineStr">
-        <is>
-          <t>Opadry Yellow 03F620190(IH,Colorcon)</t>
-        </is>
-      </c>
-      <c r="D112" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E112" s="8" t="inlineStr">
-        <is>
-          <t>2025-03-18</t>
-        </is>
-      </c>
-      <c r="F112" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G112" s="8" t="n">
-        <v>462</v>
-      </c>
-      <c r="H112" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="I112" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J112" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K112" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B113" s="8" t="n">
-        <v>1300181</v>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t>Opadry QX 321A120007 Yellow(칼라콘,별규)</t>
-        </is>
-      </c>
-      <c r="D113" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E113" s="8" t="inlineStr">
-        <is>
-          <t>2025-03-25</t>
-        </is>
-      </c>
-      <c r="F113" s="8" t="n">
-        <v>391</v>
-      </c>
-      <c r="G113" s="8" t="n">
-        <v>455</v>
-      </c>
-      <c r="H113" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="I113" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J113" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K113" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="18" customHeight="1">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B114" s="8" t="n">
-        <v>1000202</v>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t>0.1% Cyanocobalamin(Ningxia)</t>
-        </is>
-      </c>
-      <c r="D114" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E114" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-14</t>
-        </is>
-      </c>
-      <c r="F114" s="8" t="n">
-        <v>72</v>
-      </c>
-      <c r="G114" s="8" t="n">
-        <v>435</v>
-      </c>
-      <c r="H114" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I114" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J114" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K114" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B115" s="8" t="n">
-        <v>1000367</v>
-      </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>Opadry OY-S-29019</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="inlineStr">
-        <is>
-          <t>3,4</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-15</t>
-        </is>
-      </c>
-      <c r="F115" s="8" t="n">
-        <v>79</v>
-      </c>
-      <c r="G115" s="8" t="n">
-        <v>434</v>
-      </c>
-      <c r="H115" s="8" t="n">
-        <v>133.3</v>
-      </c>
-      <c r="I115" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J115" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K115" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="18" customHeight="1">
-      <c r="A116" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B116" s="8" t="n">
-        <v>1301203</v>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>Opadry AMB II 88A610005 GREEN (별규,칼라콘)</t>
-        </is>
-      </c>
-      <c r="D116" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E116" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-16</t>
-        </is>
-      </c>
-      <c r="F116" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="G116" s="8" t="n">
-        <v>433</v>
-      </c>
-      <c r="H116" s="8" t="n">
-        <v>175</v>
-      </c>
-      <c r="I116" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J116" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K116" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B117" s="8" t="n">
-        <v>1300614</v>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>Human serum albumin(세관폐기)</t>
-        </is>
-      </c>
-      <c r="D117" s="8" t="inlineStr">
-        <is>
-          <t>1,4</t>
-        </is>
-      </c>
-      <c r="E117" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-28</t>
-        </is>
-      </c>
-      <c r="F117" s="8" t="n">
-        <v>75</v>
-      </c>
-      <c r="G117" s="8" t="n">
-        <v>421</v>
-      </c>
-      <c r="H117" s="8" t="n">
-        <v>31200</v>
-      </c>
-      <c r="I117" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J117" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K117" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B118" s="8" t="n">
-        <v>1300949</v>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>Opadry Pink 03F640111(IH,칼라콘)</t>
-        </is>
-      </c>
-      <c r="D118" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E118" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-28</t>
-        </is>
-      </c>
-      <c r="F118" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G118" s="8" t="n">
-        <v>421</v>
-      </c>
-      <c r="H118" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="I118" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J118" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K118" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B119" s="8" t="n">
-        <v>1301322</v>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>Oxymetazoline HCl(USP,CTX)</t>
-        </is>
-      </c>
-      <c r="D119" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t>2025-04-30</t>
-        </is>
-      </c>
-      <c r="F119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G119" s="8" t="n">
-        <v>419</v>
-      </c>
-      <c r="H119" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="I119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J119" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K119" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t>⚪ 발주중단의심</t>
-        </is>
-      </c>
-      <c r="B120" s="8" t="n">
-        <v>1300438</v>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>오파드라이 20A680000 칼라콘</t>
-        </is>
-      </c>
-      <c r="D120" s="8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E120" s="8" t="inlineStr">
-        <is>
-          <t>2025-05-29</t>
-        </is>
-      </c>
-      <c r="F120" s="8" t="n">
-        <v>249</v>
-      </c>
-      <c r="G120" s="8" t="n">
-        <v>390</v>
-      </c>
-      <c r="H120" s="8" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="I120" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J120" s="8" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K120" s="8" t="inlineStr">
-        <is>
-          <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K120"/>
+  <autoFilter ref="A1:K102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6377,31 +5423,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>🆕 신규품목</t>
+          <t>🔴 발주확인</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>🔴 발주확인</t>
+          <t>🟢 정상</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>🟢 정상</t>
+          <t>🆕 신규품목</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
excel update 2026-06-23 14:48
</commit_message>
<xml_diff>
--- a/order_result.xlsx
+++ b/order_result.xlsx
@@ -11,7 +11,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'발주확인대상'!$A$1:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'발주확인대상'!$A$1:$J$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -557,11 +557,6 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>수량달성률</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
           <t>비고</t>
         </is>
       </c>
@@ -604,11 +599,6 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
           <t>간격 358일 경과(평균 178일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -651,11 +641,6 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
           <t>간격 330일 경과(평균 106일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -698,11 +683,6 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
           <t>간격 303일 경과(평균 57일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -745,11 +725,6 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
           <t>간격 300일 경과(평균 51일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -792,11 +767,6 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
           <t>간격 300일 경과(평균 51일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -839,11 +809,6 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
           <t>간격 292일 경과(평균 39일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -886,11 +851,6 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
           <t>간격 291일 경과(평균 63일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -933,11 +893,6 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
           <t>간격 288일 경과(평균 122일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -980,11 +935,6 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
           <t>간격 235일 경과(평균 27일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1027,11 +977,6 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
           <t>간격 235일 경과(평균 46일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1074,11 +1019,6 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
           <t>간격 210일 경과(평균 63일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1121,11 +1061,6 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
           <t>간격 200일 경과(평균 137일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1168,11 +1103,6 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
           <t>간격 197일 경과(평균 95일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1215,11 +1145,6 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
           <t>간격 197일 경과(평균 71일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1262,11 +1187,6 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
           <t>간격 186일 경과(평균 79일) + 올해 수량 연평균의 0% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1309,11 +1229,6 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>21%</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
           <t>간격 145일 경과(평균 54일) + 올해 수량 연평균의 21% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1356,11 +1271,6 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
           <t>간격 95일 경과(평균 23일) + 올해 수량 연평균의 9% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1403,11 +1313,6 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>31%</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
           <t>간격 56일 경과(평균 30일) + 올해 수량 연평균의 31% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1450,11 +1355,6 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
           <t>간격 56일 경과(평균 37일) + 올해 수량 연평균의 17% — 즉시 확인 필요</t>
         </is>
       </c>
@@ -1462,7 +1362,7 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
@@ -1497,11 +1397,6 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1509,7 +1404,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -1544,11 +1439,6 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1556,7 +1446,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
@@ -1591,11 +1481,6 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1603,7 +1488,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
@@ -1638,11 +1523,6 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1650,7 +1530,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
@@ -1685,11 +1565,6 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1697,7 +1572,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
@@ -1732,11 +1607,6 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 0% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1744,7 +1614,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
@@ -1779,11 +1649,6 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 67% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1791,7 +1656,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
@@ -1826,11 +1691,6 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 67% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1838,7 +1698,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -1873,11 +1733,6 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>22%</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 22% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1885,7 +1740,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -1920,11 +1775,6 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>77%</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 77% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1932,7 +1782,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
@@ -1967,11 +1817,6 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 25% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -1979,7 +1824,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
@@ -2014,11 +1859,6 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 17% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2026,7 +1866,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -2061,11 +1901,6 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 50% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2073,7 +1908,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
@@ -2108,11 +1943,6 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>29%</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 29% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2120,7 +1950,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -2155,11 +1985,6 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>55%</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 55% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2167,7 +1992,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
@@ -2202,11 +2027,6 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>43%</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 43% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2214,7 +2034,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -2249,11 +2069,6 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>7%</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 7% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2261,7 +2076,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
@@ -2296,11 +2111,6 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>51%</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 51% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2308,7 +2118,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
@@ -2343,11 +2153,6 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>42%</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 42% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2355,7 +2160,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
@@ -2390,11 +2195,6 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 25% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2402,7 +2202,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
@@ -2437,11 +2237,6 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 50% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2449,7 +2244,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
@@ -2484,11 +2279,6 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>12%</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 12% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2496,7 +2286,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -2531,11 +2321,6 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>53%</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 53% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2543,7 +2328,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
@@ -2578,11 +2363,6 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>31%</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 31% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2590,7 +2370,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -2625,11 +2405,6 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>62%</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 62% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2637,7 +2412,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
@@ -2672,11 +2447,6 @@
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>66%</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 66% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2684,7 +2454,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -2719,11 +2489,6 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 10% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2731,7 +2496,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
@@ -2766,11 +2531,6 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>36%</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 36% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2778,7 +2538,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
@@ -2813,11 +2573,6 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>45%</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 45% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2825,7 +2580,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
@@ -2860,11 +2615,6 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>75%</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 75% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2872,7 +2622,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
@@ -2907,11 +2657,6 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>33%</t>
-        </is>
-      </c>
-      <c r="K51" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 33% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -2919,7 +2664,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
@@ -2954,11 +2699,6 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="K52" s="4" t="inlineStr">
-        <is>
           <t>발주 간격은 정상이나 올해 수량이 연평균의 20% — 수량 부족 확인 필요</t>
         </is>
       </c>
@@ -3001,11 +2741,6 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>112%</t>
-        </is>
-      </c>
-      <c r="K53" s="5" t="inlineStr">
-        <is>
           <t>간격 68일 경과(평균 33일)이나 올해 수량 연평균의 112% — 수량 기준 이상 없음</t>
         </is>
       </c>
@@ -3048,11 +2783,6 @@
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>187%</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr">
-        <is>
           <t>간격 75일 경과(평균 334일), 올해 수량 연평균의 187% — 이상 없음</t>
         </is>
       </c>
@@ -3095,11 +2825,6 @@
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>103%</t>
-        </is>
-      </c>
-      <c r="K55" s="6" t="inlineStr">
-        <is>
           <t>간격 41일 경과(평균 106일), 올해 수량 연평균의 103% — 이상 없음</t>
         </is>
       </c>
@@ -3142,11 +2867,6 @@
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>92%</t>
-        </is>
-      </c>
-      <c r="K56" s="6" t="inlineStr">
-        <is>
           <t>간격 35일 경과(평균 112일), 올해 수량 연평균의 92% — 이상 없음</t>
         </is>
       </c>
@@ -3189,11 +2909,6 @@
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>107%</t>
-        </is>
-      </c>
-      <c r="K57" s="6" t="inlineStr">
-        <is>
           <t>간격 35일 경과(평균 254일), 올해 수량 연평균의 107% — 이상 없음</t>
         </is>
       </c>
@@ -3236,11 +2951,6 @@
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>110%</t>
-        </is>
-      </c>
-      <c r="K58" s="6" t="inlineStr">
-        <is>
           <t>간격 35일 경과(평균 151일), 올해 수량 연평균의 110% — 이상 없음</t>
         </is>
       </c>
@@ -3283,11 +2993,6 @@
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>215%</t>
-        </is>
-      </c>
-      <c r="K59" s="6" t="inlineStr">
-        <is>
           <t>간격 28일 경과(평균 104일), 올해 수량 연평균의 215% — 이상 없음</t>
         </is>
       </c>
@@ -3330,11 +3035,6 @@
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K60" s="6" t="inlineStr">
-        <is>
           <t>간격 21일 경과(평균 83일), 올해 수량 연평균의 80% — 이상 없음</t>
         </is>
       </c>
@@ -3377,11 +3077,6 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>135%</t>
-        </is>
-      </c>
-      <c r="K61" s="6" t="inlineStr">
-        <is>
           <t>간격 13일 경과(평균 145일), 올해 수량 연평균의 135% — 이상 없음</t>
         </is>
       </c>
@@ -3424,11 +3119,6 @@
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>118%</t>
-        </is>
-      </c>
-      <c r="K62" s="6" t="inlineStr">
-        <is>
           <t>간격 12일 경과(평균 119일), 올해 수량 연평균의 118% — 이상 없음</t>
         </is>
       </c>
@@ -3471,11 +3161,6 @@
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>90%</t>
-        </is>
-      </c>
-      <c r="K63" s="6" t="inlineStr">
-        <is>
           <t>간격 12일 경과(평균 67일), 올해 수량 연평균의 90% — 이상 없음</t>
         </is>
       </c>
@@ -3518,11 +3203,6 @@
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>96%</t>
-        </is>
-      </c>
-      <c r="K64" s="6" t="inlineStr">
-        <is>
           <t>간격 12일 경과(평균 65일), 올해 수량 연평균의 96% — 이상 없음</t>
         </is>
       </c>
@@ -3571,11 +3251,6 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K65" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3624,11 +3299,6 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K66" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3677,11 +3347,6 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K67" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3730,11 +3395,6 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K68" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3783,11 +3443,6 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K69" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3836,11 +3491,6 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K70" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3889,11 +3539,6 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K71" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3942,11 +3587,6 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K72" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -3995,11 +3635,6 @@
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K73" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -4048,11 +3683,6 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K74" s="7" t="inlineStr">
-        <is>
           <t>과거 3개년 이력 없는 신규 품목</t>
         </is>
       </c>
@@ -4060,7 +3690,7 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B75" s="8" t="n">
@@ -4095,11 +3725,6 @@
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K75" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4107,7 +3732,7 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B76" s="8" t="n">
@@ -4142,11 +3767,6 @@
       </c>
       <c r="J76" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K76" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4154,7 +3774,7 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B77" s="8" t="n">
@@ -4189,11 +3809,6 @@
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K77" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4201,7 +3816,7 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B78" s="8" t="n">
@@ -4236,11 +3851,6 @@
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K78" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4248,7 +3858,7 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B79" s="8" t="n">
@@ -4283,11 +3893,6 @@
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K79" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4295,7 +3900,7 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B80" s="8" t="n">
@@ -4330,11 +3935,6 @@
       </c>
       <c r="J80" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K80" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4342,7 +3942,7 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B81" s="8" t="n">
@@ -4377,11 +3977,6 @@
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K81" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4389,7 +3984,7 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B82" s="8" t="n">
@@ -4424,11 +4019,6 @@
       </c>
       <c r="J82" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K82" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4436,7 +4026,7 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B83" s="8" t="n">
@@ -4471,11 +4061,6 @@
       </c>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K83" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4483,7 +4068,7 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B84" s="8" t="n">
@@ -4518,11 +4103,6 @@
       </c>
       <c r="J84" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K84" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4530,7 +4110,7 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B85" s="8" t="n">
@@ -4565,11 +4145,6 @@
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K85" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4577,7 +4152,7 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B86" s="8" t="n">
@@ -4612,11 +4187,6 @@
       </c>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K86" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4624,7 +4194,7 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B87" s="8" t="n">
@@ -4659,11 +4229,6 @@
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K87" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4671,7 +4236,7 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B88" s="8" t="n">
@@ -4706,11 +4271,6 @@
       </c>
       <c r="J88" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K88" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4718,7 +4278,7 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B89" s="8" t="n">
@@ -4753,11 +4313,6 @@
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K89" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4765,7 +4320,7 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B90" s="8" t="n">
@@ -4800,11 +4355,6 @@
       </c>
       <c r="J90" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K90" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4812,7 +4362,7 @@
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B91" s="8" t="n">
@@ -4847,11 +4397,6 @@
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K91" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4859,7 +4404,7 @@
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B92" s="8" t="n">
@@ -4894,11 +4439,6 @@
       </c>
       <c r="J92" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K92" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4906,7 +4446,7 @@
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
@@ -4941,11 +4481,6 @@
       </c>
       <c r="J93" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K93" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -4953,7 +4488,7 @@
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B94" s="8" t="n">
@@ -4988,11 +4523,6 @@
       </c>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K94" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5000,7 +4530,7 @@
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B95" s="8" t="n">
@@ -5035,11 +4565,6 @@
       </c>
       <c r="J95" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K95" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5047,7 +4572,7 @@
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B96" s="8" t="n">
@@ -5082,11 +4607,6 @@
       </c>
       <c r="J96" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K96" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5094,7 +4614,7 @@
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B97" s="8" t="n">
@@ -5129,11 +4649,6 @@
       </c>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K97" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5141,7 +4656,7 @@
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B98" s="8" t="n">
@@ -5176,11 +4691,6 @@
       </c>
       <c r="J98" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K98" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5188,7 +4698,7 @@
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B99" s="8" t="n">
@@ -5223,11 +4733,6 @@
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K99" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5235,7 +4740,7 @@
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B100" s="8" t="n">
@@ -5270,11 +4775,6 @@
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K100" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5282,7 +4782,7 @@
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B101" s="8" t="n">
@@ -5317,11 +4817,6 @@
       </c>
       <c r="J101" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K101" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
@@ -5329,7 +4824,7 @@
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B102" s="8" t="n">
@@ -5364,17 +4859,12 @@
       </c>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="K102" s="8" t="inlineStr">
-        <is>
           <t>최근 1년간 발주 없음 — 발주 중단 여부 확인</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K102"/>
+  <autoFilter ref="A1:J102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5403,7 +4893,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>🟠 수량부족주의</t>
+          <t>🟠 수량확인</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -5413,7 +4903,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>⚪ 발주중단의심</t>
+          <t>⚪ 발주없음</t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>